<commit_message>
Enable ec002 with confirmed maintenance and miscellaneous budget locks
</commit_message>
<xml_diff>
--- a/data/source/Event.xlsx
+++ b/data/source/Event.xlsx
@@ -396,7 +396,7 @@
           <t>option 2 result</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="0" t="inlineStr">
         <is>
           <t>enabled</t>
         </is>
@@ -431,7 +431,7 @@
           <t>每片上座率*0.67</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -466,7 +466,7 @@
           <t>每片上座率*0.33；其它支出強制鎖定為100,000</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -505,7 +505,7 @@
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="n"/>
       <c r="J4" s="2" t="n"/>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -544,7 +544,7 @@
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="n"/>
       <c r="J5" s="2" t="n"/>
-      <c r="K5" t="inlineStr">
+      <c r="K5" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -579,7 +579,7 @@
           <t>雜支強制鎖定為1,000,000；每片上座率*0.33</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K6" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -618,7 +618,7 @@
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="n"/>
       <c r="J7" s="2" t="n"/>
-      <c r="K7" t="inlineStr">
+      <c r="K7" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -657,7 +657,7 @@
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
       <c r="J8" s="2" t="n"/>
-      <c r="K8" t="inlineStr">
+      <c r="K8" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -692,7 +692,7 @@
           <t>每片上座率*0.1；硬體維護強制鎖定為50,000</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K9" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -747,7 +747,7 @@
           <t>每片上座率*0.01</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K10" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -782,7 +782,7 @@
           <t>每片上座率*0.33</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K11" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -817,7 +817,7 @@
           <t>連四週每片上座率*1.2</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K12" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -856,7 +856,7 @@
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="n"/>
       <c r="J13" s="2" t="n"/>
-      <c r="K13" t="inlineStr">
+      <c r="K13" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -895,7 +895,7 @@
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="n"/>
-      <c r="K14" t="inlineStr">
+      <c r="K14" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -950,7 +950,7 @@
           <t>所有收入歸0；人力預算、硬體維護以最低值支出</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K15" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1005,7 +1005,7 @@
           <t>人力預算強制鎖定為(廳數+1)*12000</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K16" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1040,7 +1040,7 @@
           <t>人力預算強制鎖定為(廳數+1)*12,000</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K17" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="G18" s="2" t="n"/>
-      <c r="K18" t="inlineStr">
+      <c r="K18" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1111,7 +1111,7 @@
           <t>硬體維護強加200,000</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K19" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1166,7 +1166,7 @@
           <t>unchanged</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="K20" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1201,7 +1201,7 @@
           <t>發撫慰金，財報人事支出強制加20,000</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="K21" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1240,7 +1240,7 @@
       <c r="H22" s="2" t="n"/>
       <c r="I22" s="2" t="n"/>
       <c r="J22" s="2" t="n"/>
-      <c r="K22" t="inlineStr">
+      <c r="K22" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1275,7 +1275,7 @@
           <t>每片上座率*4；人力預算強制鎖定為(廳數+1)*12,000</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="K23" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1330,7 +1330,7 @@
           <t>人事額外支出20000；普通片上座率*1.1</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="K24" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1385,7 +1385,7 @@
           <t>人事額外支出20000；普通片上座率*1.1</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="K25" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1420,7 +1420,7 @@
           <t>當週主打片上座率歸0</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K26" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1452,16 +1452,16 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>其它支出強制鎖定為100,000；雜支強制鎖定為20,000</t>
+          <t>硬體強制鎖定為100,000；雜支強制鎖定為20,000</t>
         </is>
       </c>
       <c r="G27" s="2" t="n"/>
       <c r="H27" s="2" t="n"/>
       <c r="I27" s="2" t="n"/>
       <c r="J27" s="2" t="n"/>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>N</t>
+      <c r="K27" s="0" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1514,7 @@
           <t>unchanged</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="K28" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1569,7 +1569,7 @@
           <t>unchanged</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="K29" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1608,7 +1608,7 @@
       <c r="H30" s="2" t="n"/>
       <c r="I30" s="2" t="n"/>
       <c r="J30" s="2" t="n"/>
-      <c r="K30" t="inlineStr">
+      <c r="K30" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1643,7 +1643,7 @@
           <t>雜支強制鎖定為20,000</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="K31" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1698,7 +1698,7 @@
           <t>unchanged</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="K32" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1733,7 +1733,7 @@
           <t>每片上座率*0.67</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="K33" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1768,7 +1768,7 @@
           <t>停車場收入歸0</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="K34" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1803,7 +1803,7 @@
           <t>財報硬體項目強制+60,000,000；12週後戲院簡介出現一個IMAX廳，首週可設IMAX票價（該週彈出視窗確認票價）</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="K35" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1838,7 +1838,7 @@
           <t>財報硬體項目強制+40,000,000；12週後戲院簡介出現一個4DX廳，首週可設4DX票價（該週彈出視窗確認票價）</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="K36" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1873,7 +1873,7 @@
           <t>財報硬體項目強制+(100,000*影廳數)；接下來一週停業全部收入歸0，再接下來24週全部上座率*1.2</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="K37" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1912,7 +1912,7 @@
       <c r="H38" s="2" t="n"/>
       <c r="I38" s="2" t="n"/>
       <c r="J38" s="2" t="n"/>
-      <c r="K38" t="inlineStr">
+      <c r="K38" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1947,7 +1947,7 @@
           <t>財報硬體項目強制+10,000,000，下一週起IMAX廳從廳數資料消失</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="K39" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1982,7 +1982,7 @@
           <t>財報硬體項目強制+5,000,000，下一週起4DX廳從廳數資料消失</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
+      <c r="K40" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2037,7 +2037,7 @@
           <t>unchanged</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="K41" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2072,7 +2072,7 @@
           <t>連四週商品成本強制加150,000，連四週人事強制加50,000；連四週餐飲收入加300,000</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="K42" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2111,7 +2111,7 @@
       <c r="H43" s="2" t="n"/>
       <c r="I43" s="2" t="n"/>
       <c r="J43" s="2" t="n"/>
-      <c r="K43" t="inlineStr">
+      <c r="K43" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2146,7 +2146,7 @@
           <t>餐飲收入歸0</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="K44" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2181,7 +2181,7 @@
           <t>當週上座率*0.1，海報訂製量鎖定為0</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="K45" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2216,7 +2216,7 @@
           <t>當週上座率*0.1，公仔訂製量鎖定為0</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="K46" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2251,7 +2251,7 @@
           <t>當週主打片上座率*0.1</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="K47" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2286,7 +2286,7 @@
           <t>當週主打片上座率直達100%</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
+      <c r="K48" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2325,7 +2325,7 @@
       <c r="H49" s="2" t="n"/>
       <c r="I49" s="2" t="n"/>
       <c r="J49" s="2" t="n"/>
-      <c r="K49" t="inlineStr">
+      <c r="K49" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2364,7 +2364,7 @@
       <c r="H50" s="2" t="n"/>
       <c r="I50" s="2" t="n"/>
       <c r="J50" s="2" t="n"/>
-      <c r="K50" t="inlineStr">
+      <c r="K50" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2419,7 +2419,7 @@
           <t>unchanged</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr">
+      <c r="K51" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2474,7 +2474,7 @@
           <t>unchanged</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
+      <c r="K52" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2529,7 +2529,7 @@
           <t>unchanged</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
+      <c r="K53" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2584,7 +2584,7 @@
           <t>unchanged</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
+      <c r="K54" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2639,7 +2639,7 @@
           <t>unchanged</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr">
+      <c r="K55" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2674,7 +2674,7 @@
           <t>當週主打片上座率*0.2</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr">
+      <c r="K56" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2709,7 +2709,7 @@
           <t>當週主打片上座率*0.2</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr">
+      <c r="K57" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2744,7 +2744,7 @@
           <t>每片上座率*2</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr">
+      <c r="K58" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2779,7 +2779,7 @@
           <t>片名含「鬼」字上座率*3</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr">
+      <c r="K59" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2814,7 +2814,7 @@
           <t>當週主打片上座率直達100%</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr">
+      <c r="K60" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2849,7 +2849,7 @@
           <t>當週主打片上座率*2</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr">
+      <c r="K61" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2884,7 +2884,7 @@
           <t>當週主打片上座率*2</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr">
+      <c r="K62" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2919,7 +2919,7 @@
           <t>上映中的MV0004,MV0005,MV0006上座率*3</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr">
+      <c r="K63" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2954,7 +2954,7 @@
           <t>上映中的MV0023,MV0024上座率*3</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr">
+      <c r="K64" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2989,7 +2989,7 @@
           <t>上映中的MV0391上座率*3</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr">
+      <c r="K65" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3024,7 +3024,7 @@
           <t>上映中的MV0387上座率*3</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr">
+      <c r="K66" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3059,7 +3059,7 @@
           <t>上映中的MV0469上座率*3</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr">
+      <c r="K67" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3094,7 +3094,7 @@
           <t>SR017電影上座率*2</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr">
+      <c r="K68" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3129,7 +3129,7 @@
           <t>SR013電影上座率*5</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr">
+      <c r="K69" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3164,7 +3164,7 @@
           <t>average film上座率*1.5</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr">
+      <c r="K70" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3199,7 +3199,7 @@
           <t>unchanged</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr">
+      <c r="K71" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3234,7 +3234,7 @@
           <t>當週主打片上座率直達100%</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr">
+      <c r="K72" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3269,7 +3269,7 @@
           <t>當週特別場出售人數基數變200人</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr">
+      <c r="K73" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3308,7 +3308,7 @@
       <c r="H74" s="2" t="n"/>
       <c r="I74" s="2" t="n"/>
       <c r="J74" s="2" t="n"/>
-      <c r="K74" t="inlineStr">
+      <c r="K74" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3347,7 +3347,7 @@
       <c r="H75" s="2" t="n"/>
       <c r="I75" s="2" t="n"/>
       <c r="J75" s="2" t="n"/>
-      <c r="K75" t="inlineStr">
+      <c r="K75" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3402,7 +3402,7 @@
           <t>所有收入歸0；人力預算、硬體維護以最低值支出</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr">
+      <c r="K76" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3437,7 +3437,7 @@
           <t>跳至年度會議結算成績；按鍵「下一年度」變成「退出」</t>
         </is>
       </c>
-      <c r="K77" t="inlineStr">
+      <c r="K77" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3472,7 +3472,7 @@
           <t>其它收入=總座位數*1000000*租金location係數；切換承租</t>
         </is>
       </c>
-      <c r="K78" t="inlineStr">
+      <c r="K78" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3507,7 +3507,7 @@
           <t>租金隨機加10%至20%</t>
         </is>
       </c>
-      <c r="K79" t="inlineStr">
+      <c r="K79" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3542,7 +3542,7 @@
           <t>再過24週跳至年度會議結算成績；按鍵「下一年度」變成「退出」</t>
         </is>
       </c>
-      <c r="K80" t="inlineStr">
+      <c r="K80" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3577,7 +3577,7 @@
           <t>再過4週跳至年度會議結算成績；按鍵「下一年度」變成「退出」</t>
         </is>
       </c>
-      <c r="K81" t="inlineStr">
+      <c r="K81" s="0" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>